<commit_message>
Fix actual center-target coaching; update First Bell production plan, evidence gates and exact authored workbook
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R41863cfd10cc4aef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rbbacf1e3250e4d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="Raa28e057d2bb4d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R453409fbb5c9478d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="Raa0d72a210d1425e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="Rb91a47b04f4d4605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rab5f026d96b64b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R62405f211b114cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R19de5b7fac5b4206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R249b587ac3e44e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="Rd1e2ed859aae4e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R2ce5060854cf48fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -203,28 +203,28 @@
   <x:dxfs count="6">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEFE8"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE6D8"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDF1F5"/>
         </x:patternFill>
       </x:fill>
@@ -235,7 +235,7 @@
         <x:color rgb="FF8A2D28"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAE3DF"/>
         </x:patternFill>
       </x:fill>
@@ -246,7 +246,7 @@
         <x:color rgb="FF8A2D28"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAE3DF"/>
         </x:patternFill>
       </x:fill>
@@ -572,7 +572,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.9.0 / Pilgrim's Rest / 2026-09-12. AAA-level finish is the aspiration, not a certified label or a promised budget. This workbook maps concrete quality gates without claiming that a completed-task count measures game quality.</x:v>
+        <x:v>v0.10.0 / First Bell / 2026-09-12. AAA-level finish is the aspiration, not a certified label or promised budget. Concrete quality gates remain separate from feature counts.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -718,7 +718,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>This release closes saved-expedition software continuity and roadmap drift. The next proposed feature work is V49 onboarding and V50 coordinated encounters, then V51 first boss and V52 route grammar, integrated in V76.</x:v>
+        <x:v>This release adds ten guided archery lessons and the optional Bellkeeper Oath: three connected encounters, a three-phase boss, recovery beats and saved continuation. V49-V52 and V76 remain Partial until their broader human, hardware and production gates are met.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -846,7 +846,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: 47e37e6b583120c17dc1b032477c63172001e0515a2f0b9d8bb7f74acb6952c7</x:v>
+        <x:v>Canonical JSON SHA-256: 8328c5cd8170c612c81c810eeeae531db22beffa97a4d5e7a67ae3c6733c490a</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -1252,9 +1252,7 @@
       <x:c r="K9" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L9" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L9" s="6" t="str"/>
       <x:c r="M9" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -1387,9 +1385,7 @@
       <x:c r="K12" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L12" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L12" s="6" t="str"/>
       <x:c r="M12" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -1431,12 +1427,8 @@
       <x:c r="K13" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
-      <x:c r="L13" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M13" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L13" s="6" t="str"/>
+      <x:c r="M13" s="6" t="str"/>
       <x:c r="N13" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -1475,12 +1467,8 @@
       <x:c r="K14" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
-      <x:c r="L14" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M14" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L14" s="6" t="str"/>
+      <x:c r="M14" s="6" t="str"/>
       <x:c r="N14" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -1519,12 +1507,8 @@
       <x:c r="K15" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
-      <x:c r="L15" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M15" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L15" s="6" t="str"/>
+      <x:c r="M15" s="6" t="str"/>
       <x:c r="N15" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -1659,9 +1643,7 @@
         <x:v>encounters.js
 bestiary.js</x:v>
       </x:c>
-      <x:c r="M18" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="M18" s="6" t="str"/>
       <x:c r="N18" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/encounters.js</x:v>
       </x:c>
@@ -1704,9 +1686,7 @@
         <x:v>resonance-audio.js
 dominion-art.js</x:v>
       </x:c>
-      <x:c r="M19" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="M19" s="6" t="str"/>
       <x:c r="N19" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/resonance-audio.js</x:v>
       </x:c>
@@ -1792,12 +1772,8 @@
       <x:c r="K21" s="6" t="str">
         <x:v>Not closed.</x:v>
       </x:c>
-      <x:c r="L21" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M21" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L21" s="6" t="str"/>
+      <x:c r="M21" s="6" t="str"/>
       <x:c r="N21" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -1836,12 +1812,8 @@
       <x:c r="K22" s="6" t="str">
         <x:v>Not closed.</x:v>
       </x:c>
-      <x:c r="L22" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M22" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L22" s="6" t="str"/>
+      <x:c r="M22" s="6" t="str"/>
       <x:c r="N22" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -1880,9 +1852,7 @@
       <x:c r="K23" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L23" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L23" s="6" t="str"/>
       <x:c r="M23" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -1924,9 +1894,7 @@
       <x:c r="K24" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L24" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L24" s="6" t="str"/>
       <x:c r="M24" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -1968,9 +1936,7 @@
       <x:c r="K25" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L25" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L25" s="6" t="str"/>
       <x:c r="M25" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2108,9 +2074,7 @@
         <x:v>tests/unchained-combat.py
 tests/browser.py</x:v>
       </x:c>
-      <x:c r="M28" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="M28" s="6" t="str"/>
       <x:c r="N28" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/unchained-combat.py</x:v>
       </x:c>
@@ -2149,12 +2113,8 @@
       <x:c r="K29" s="6" t="str">
         <x:v>Not closed.</x:v>
       </x:c>
-      <x:c r="L29" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M29" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L29" s="6" t="str"/>
+      <x:c r="M29" s="6" t="str"/>
       <x:c r="N29" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -2239,9 +2199,7 @@
       <x:c r="K31" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L31" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L31" s="6" t="str"/>
       <x:c r="M31" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2283,9 +2241,7 @@
       <x:c r="K32" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L32" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L32" s="6" t="str"/>
       <x:c r="M32" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2327,9 +2283,7 @@
       <x:c r="K33" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L33" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L33" s="6" t="str"/>
       <x:c r="M33" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2371,9 +2325,7 @@
       <x:c r="K34" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L34" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L34" s="6" t="str"/>
       <x:c r="M34" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2418,9 +2370,7 @@
       <x:c r="L35" s="6" t="str">
         <x:v>RESONANT-HUNT.md</x:v>
       </x:c>
-      <x:c r="M35" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="M35" s="6" t="str"/>
       <x:c r="N35" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/RESONANT-HUNT.md</x:v>
       </x:c>
@@ -2459,9 +2409,7 @@
       <x:c r="K36" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L36" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L36" s="6" t="str"/>
       <x:c r="M36" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2503,9 +2451,7 @@
       <x:c r="K37" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L37" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L37" s="6" t="str"/>
       <x:c r="M37" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2547,9 +2493,7 @@
       <x:c r="K38" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L38" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L38" s="6" t="str"/>
       <x:c r="M38" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2591,9 +2535,7 @@
       <x:c r="K39" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L39" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L39" s="6" t="str"/>
       <x:c r="M39" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2639,9 +2581,7 @@
         <x:v>dominions-world.js
 HOLLOW-DOMINIONS.md</x:v>
       </x:c>
-      <x:c r="M40" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="M40" s="6" t="str"/>
       <x:c r="N40" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominions-world.js</x:v>
       </x:c>
@@ -2680,12 +2620,8 @@
       <x:c r="K41" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
-      <x:c r="L41" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M41" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L41" s="6" t="str"/>
+      <x:c r="M41" s="6" t="str"/>
       <x:c r="N41" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -2724,9 +2660,7 @@
       <x:c r="K42" s="6" t="str">
         <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
       </x:c>
-      <x:c r="L42" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
+      <x:c r="L42" s="6" t="str"/>
       <x:c r="M42" s="6" t="str">
         <x:v>Baseline through 0.6.0</x:v>
       </x:c>
@@ -2768,12 +2702,8 @@
       <x:c r="K43" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
-      <x:c r="L43" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M43" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L43" s="6" t="str"/>
+      <x:c r="M43" s="6" t="str"/>
       <x:c r="N43" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3245,7 +3175,7 @@
         <x:v>First ten minutes: playable physical onboarding</x:v>
       </x:c>
       <x:c r="C54" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D54" s="6" t="str">
         <x:v>P0</x:v>
@@ -3269,16 +3199,17 @@
         <x:v>A new player can learn nock/draw, cancel, reload, shield, Blink, shard step, pickups and quiver in either handedness, then enter a short scored encounter. Record completion, confusion and fatigue.</x:v>
       </x:c>
       <x:c r="K54" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Ten playable lessons now verify actual outcomes, with device-specific hints and a spatial Quest coach. Skips are recorded separately. Software-only: first-user confusion, reversed-hand ergonomics and fatigue remain to be measured.</x:v>
       </x:c>
       <x:c r="L54" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
+        <x:v>first-bell.js
+tests/first-bell-browser.py</x:v>
       </x:c>
       <x:c r="M54" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
+        <x:v>0.10.0 First Bell</x:v>
       </x:c>
       <x:c r="N54" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/first-bell.js</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="124" customHeight="1">
@@ -3289,7 +3220,7 @@
         <x:v>Encounter director with fair threat and recovery budgets</x:v>
       </x:c>
       <x:c r="C55" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D55" s="6" t="str">
         <x:v>P0</x:v>
@@ -3313,16 +3244,18 @@
         <x:v>Coordinate telegraphed melee/ranged attacks, limit unavoidable overlap and offscreen attacks, preserve escape routes and add recovery beats. Replay fixed-seed stress encounters.</x:v>
       </x:c>
       <x:c r="K55" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>The optional Oath coordinates three staged encounters with front-hemisphere initiation, bolt/windup budgets and recovery supplies. The original Endless mode is unchanged. Broad seed/human difficulty evaluation remains open.</x:v>
       </x:c>
       <x:c r="L55" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
+        <x:v>oath-model.js
+tests/oath.test.cjs
+tests/first-bell-browser.py</x:v>
       </x:c>
       <x:c r="M55" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
+        <x:v>0.10.0 First Bell</x:v>
       </x:c>
       <x:c r="N55" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="124" customHeight="1">
@@ -3333,7 +3266,7 @@
         <x:v>First signature boss: readable multi-phase duel</x:v>
       </x:c>
       <x:c r="C56" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D56" s="6" t="str">
         <x:v>P1</x:v>
@@ -3357,16 +3290,19 @@
         <x:v>An original boss changes tactics across three tested phases, uses cover/height, offers weak-point windows and has no unavoidable transition damage or restart softlock.</x:v>
       </x:c>
       <x:c r="K56" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>The Bellkeeper has three committed attack phases, armor/recovery weak points and protected transitions. Original procedural character art is implemented; production rigging, animation and human difficulty approval are not complete.</x:v>
       </x:c>
       <x:c r="L56" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
+        <x:v>oath-model.js
+first-bell.js
+tests/oath.test.cjs
+tests/first-bell-browser.py</x:v>
       </x:c>
       <x:c r="M56" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
+        <x:v>0.10.0 First Bell</x:v>
       </x:c>
       <x:c r="N56" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="124" customHeight="1">
@@ -3377,7 +3313,7 @@
         <x:v>Authored vertical-slice route grammar and route contracts</x:v>
       </x:c>
       <x:c r="C57" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D57" s="6" t="str">
         <x:v>P0</x:v>
@@ -3401,16 +3337,18 @@
         <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content.</x:v>
       </x:c>
       <x:c r="K57" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>A connected Roseglass/Ivory Crown/Ember Crown progression reuses the collision-tested 25-room world, existing stairs and alternate approaches. Three staged courts are implemented; the proposed 20-30 minute polished duration and authored connector variety are not yet measured or complete.</x:v>
       </x:c>
       <x:c r="L57" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
+        <x:v>oath-model.js
+first-bell.js
+tests/oath.test.cjs</x:v>
       </x:c>
       <x:c r="M57" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
+        <x:v>0.10.0 First Bell</x:v>
       </x:c>
       <x:c r="N57" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="124" customHeight="1">
@@ -3447,12 +3385,8 @@
       <x:c r="K58" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L58" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M58" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L58" s="6" t="str"/>
+      <x:c r="M58" s="6" t="str"/>
       <x:c r="N58" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3491,12 +3425,8 @@
       <x:c r="K59" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L59" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M59" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L59" s="6" t="str"/>
+      <x:c r="M59" s="6" t="str"/>
       <x:c r="N59" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3535,12 +3465,8 @@
       <x:c r="K60" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L60" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M60" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L60" s="6" t="str"/>
+      <x:c r="M60" s="6" t="str"/>
       <x:c r="N60" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3579,12 +3505,8 @@
       <x:c r="K61" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L61" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M61" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L61" s="6" t="str"/>
+      <x:c r="M61" s="6" t="str"/>
       <x:c r="N61" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3623,12 +3545,8 @@
       <x:c r="K62" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L62" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M62" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L62" s="6" t="str"/>
+      <x:c r="M62" s="6" t="str"/>
       <x:c r="N62" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3667,12 +3585,8 @@
       <x:c r="K63" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L63" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M63" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L63" s="6" t="str"/>
+      <x:c r="M63" s="6" t="str"/>
       <x:c r="N63" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3711,12 +3625,8 @@
       <x:c r="K64" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L64" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M64" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L64" s="6" t="str"/>
+      <x:c r="M64" s="6" t="str"/>
       <x:c r="N64" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3755,12 +3665,8 @@
       <x:c r="K65" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L65" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M65" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L65" s="6" t="str"/>
+      <x:c r="M65" s="6" t="str"/>
       <x:c r="N65" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3799,12 +3705,8 @@
       <x:c r="K66" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L66" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M66" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L66" s="6" t="str"/>
+      <x:c r="M66" s="6" t="str"/>
       <x:c r="N66" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3843,12 +3745,8 @@
       <x:c r="K67" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L67" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M67" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L67" s="6" t="str"/>
+      <x:c r="M67" s="6" t="str"/>
       <x:c r="N67" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3887,12 +3785,8 @@
       <x:c r="K68" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L68" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M68" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L68" s="6" t="str"/>
+      <x:c r="M68" s="6" t="str"/>
       <x:c r="N68" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3931,12 +3825,8 @@
       <x:c r="K69" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L69" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M69" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L69" s="6" t="str"/>
+      <x:c r="M69" s="6" t="str"/>
       <x:c r="N69" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3975,12 +3865,8 @@
       <x:c r="K70" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L70" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M70" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L70" s="6" t="str"/>
+      <x:c r="M70" s="6" t="str"/>
       <x:c r="N70" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4019,12 +3905,8 @@
       <x:c r="K71" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L71" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M71" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L71" s="6" t="str"/>
+      <x:c r="M71" s="6" t="str"/>
       <x:c r="N71" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4063,12 +3945,8 @@
       <x:c r="K72" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L72" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M72" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L72" s="6" t="str"/>
+      <x:c r="M72" s="6" t="str"/>
       <x:c r="N72" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4111,9 +3989,7 @@
         <x:v>tests/verify-live.py
 tests/launch.py</x:v>
       </x:c>
-      <x:c r="M73" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="M73" s="6" t="str"/>
       <x:c r="N73" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/verify-live.py</x:v>
       </x:c>
@@ -4152,12 +4028,8 @@
       <x:c r="K74" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L74" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M74" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L74" s="6" t="str"/>
+      <x:c r="M74" s="6" t="str"/>
       <x:c r="N74" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4196,12 +4068,8 @@
       <x:c r="K75" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L75" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M75" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L75" s="6" t="str"/>
+      <x:c r="M75" s="6" t="str"/>
       <x:c r="N75" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4240,12 +4108,8 @@
       <x:c r="K76" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L76" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M76" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L76" s="6" t="str"/>
+      <x:c r="M76" s="6" t="str"/>
       <x:c r="N76" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4284,12 +4148,8 @@
       <x:c r="K77" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L77" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M77" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L77" s="6" t="str"/>
+      <x:c r="M77" s="6" t="str"/>
       <x:c r="N77" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4328,12 +4188,8 @@
       <x:c r="K78" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L78" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M78" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L78" s="6" t="str"/>
+      <x:c r="M78" s="6" t="str"/>
       <x:c r="N78" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4372,12 +4228,8 @@
       <x:c r="K79" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L79" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M79" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L79" s="6" t="str"/>
+      <x:c r="M79" s="6" t="str"/>
       <x:c r="N79" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4416,12 +4268,8 @@
       <x:c r="K80" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L80" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
-      </x:c>
-      <x:c r="M80" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
-      </x:c>
+      <x:c r="L80" s="6" t="str"/>
+      <x:c r="M80" s="6" t="str"/>
       <x:c r="N80" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4434,7 +4282,7 @@
         <x:v>First boss and encounter slice end-to-end release</x:v>
       </x:c>
       <x:c r="C81" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D81" s="6" t="str">
         <x:v>P1</x:v>
@@ -4458,16 +4306,18 @@
         <x:v>Publish one complete integrated slice, including onboarding, traversal, encounter pacing, boss payoff and saved continuation; collect human feedback before producing additional bosses.</x:v>
       </x:c>
       <x:c r="K81" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>First Bell integrates teaching, a scored staged route, three-phase boss and checkpoint continuation in the maintained game. Source/model and native-input checks are distinct from physical hardware and human approval.</x:v>
       </x:c>
       <x:c r="L81" s="6" t="str">
-        <x:v>No completion evidence yet</x:v>
+        <x:v>FIRST-BELL.md
+tests/first-bell-browser.py
+tests/pilgrim.test.cjs</x:v>
       </x:c>
       <x:c r="M81" s="6" t="str">
-        <x:v>Future / not scheduled</x:v>
+        <x:v>0.10.0 First Bell</x:v>
       </x:c>
       <x:c r="N81" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/FIRST-BELL.md</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -4523,7 +4373,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86005719d4d14564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d611494d3364714"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4676,7 +4526,7 @@
         <x:v>Combat mastery slice</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
         <x:v>M1</x:v>
@@ -4825,7 +4675,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7d5b1a8f129479c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44c3c9b2df99468d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5214,7 +5064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f19d879ef443ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R267bdb5f9ca14712"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5560,7 +5410,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0464511bb6dd4142"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dd154f199c64b75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5936,7 +5786,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fb38ddea84740b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf74c933637714600"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Vesperfall 0.11 Rosefire: original bounded PBR, stained-light, sky, ward and landing shaders; controller settings and production workbook
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rab5f026d96b64b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R62405f211b114cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R19de5b7fac5b4206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R249b587ac3e44e3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="Rd1e2ed859aae4e3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R2ce5060854cf48fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5422c9ec86e54f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R55a7ea2099fa4869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R4b608d0afcc44efb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R78d077327f794c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R9b625fbc4c40465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R0317debfb8b54e62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -572,7 +572,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.10.0 / First Bell / 2026-09-12. AAA-level finish is the aspiration, not a certified label or promised budget. Concrete quality gates remain separate from feature counts.</x:v>
+        <x:v>v0.11.0 / Rosefire / 2026-09-12. Original gothic shaders extend the existing First Bell game. AAA-level finish remains a quality-gated aspiration, not a hardware certificate.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -846,7 +846,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: 8328c5cd8170c612c81c810eeeae531db22beffa97a4d5e7a67ae3c6733c490a</x:v>
+        <x:v>Canonical JSON SHA-256: e5fa1d8a3476502e514485305e19f4095f419ce8d165203fec6301028488fa8c</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -2631,7 +2631,7 @@
         <x:v>V37</x:v>
       </x:c>
       <x:c r="B42" s="6" t="str">
-        <x:v>Jewelglass material profiles, carved recurve and bounded spell shaders</x:v>
+        <x:v>Jewelglass and Rosefire: reflective materials, stained light and bounded shaders</x:v>
       </x:c>
       <x:c r="C42" s="6" t="str">
         <x:v>Implemented</x:v>
@@ -2646,23 +2646,30 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G42" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H42" s="6" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="I42" s="6" t="str">
-        <x:v>Preserve the established game while closing the stated acceptance gate.</x:v>
+        <x:v>Use coherent gothic light, wet stone and readable magical equipment to deepen the atmosphere without hiding combat information.</x:v>
       </x:c>
       <x:c r="J42" s="6" t="str">
-        <x:v>Native material, rebuild and emulated stereo tests plus actual served-file verification.</x:v>
+        <x:v>Publish reversible original material and shader profiles with normal/AO maps preserved, visible native-frame comparisons, controller-accessible settings, reduced-motion and passthrough-safe policies; no new gameplay or save-state writes.</x:v>
       </x:c>
       <x:c r="K42" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
-      </x:c>
-      <x:c r="L42" s="6" t="str"/>
+        <x:v>Original shader extension and automated/native rendering checks are separate from physical Quest frame-time, comfort and human art acceptance.</x:v>
+      </x:c>
+      <x:c r="L42" s="6" t="str">
+        <x:v>JEWELGLASS.md
+ROSEFIRE.md
+rosefire-shaders.js
+rosefire.js
+tests/rosefire.test.cjs
+tests/rosefire-browser.py</x:v>
+      </x:c>
       <x:c r="M42" s="6" t="str">
-        <x:v>Baseline through 0.6.0</x:v>
+        <x:v>0.11.0 Rosefire</x:v>
       </x:c>
       <x:c r="N42" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
@@ -2673,7 +2680,7 @@
         <x:v>V38</x:v>
       </x:c>
       <x:c r="B43" s="6" t="str">
-        <x:v>Measure physical Quest 3 stereo frame times for jewel reflections and shaders</x:v>
+        <x:v>Measure physical Quest 3 stereo frame times for Jewelglass and Rosefire</x:v>
       </x:c>
       <x:c r="C43" s="6" t="str">
         <x:v>Hardware QA</x:v>
@@ -2688,7 +2695,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
         <x:v>None</x:v>
@@ -2702,7 +2709,9 @@
       <x:c r="K43" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
-      <x:c r="L43" s="6" t="str"/>
+      <x:c r="L43" s="6" t="str">
+        <x:v>ROSEFIRE.md</x:v>
+      </x:c>
       <x:c r="M43" s="6" t="str"/>
       <x:c r="N43" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
@@ -4373,7 +4382,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d611494d3364714"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb18996740d4745"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4675,7 +4684,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44c3c9b2df99468d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9104c7460b48cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5064,7 +5073,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R267bdb5f9ca14712"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R096389eea6dc41da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5410,7 +5419,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dd154f199c64b75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0564014c6268424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5786,7 +5795,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf74c933637714600"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e54c835d1604ee7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>